<commit_message>
Add red line-number labels on drawings and drawings under the 询价单 table
- drawing-translate: stamp.py writes a red framed label (e.g. 询价单序号 3｜图号 …)
  into a blank area of each page, avoiding lines, table cells and highlight boxes
- supplier-rfq: place_drawings.py puts every drawing under the table and notes on
  sheet 1, sized to about one screen, anchored to move and size with cells
- drawing images are stored as palette PNGs (much smaller files)
- check_deps: numpy and pillow

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/rfq-tools/skills/supplier-rfq/templates/inquiry-template.xlsx
+++ b/plugins/rfq-tools/skills/supplier-rfq/templates/inquiry-template.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="22020" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="询价单" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="询价单" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>